<commit_message>
fix(fixtures): pin A4 in pageSetup so LibreOffice stops printing Letter
LibreOffice takes the paper size of a workbook without paperSize from the
environment: on CI and on macOS it printed Letter while our export is always
A4, so the SSIM oracle compared different pages. Environment levers were
tested and refuted (CI runs 37538750822, 37560908632, 37574459266); on macOS
there is no lever at all, libpaper is not even installed.

Paper is a property of the document, so the generator writes paperSize="9"
(A4, ECMA-376) into every sheet part after the after-hooks have repacked the
package. Our export ignores paperSize (crates/pdf takes the format from
PdfOptions::page, default A4), hence both sides now land on A4.
</commit_message>
<xml_diff>
--- a/test-fixtures/xlsx/comments-legacy.xlsx
+++ b/test-fixtures/xlsx/comments-legacy.xlsx
@@ -482,7 +482,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -499,7 +499,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>